<commit_message>
fix(mobile-bar-en): entregables regenerados tras REVISION-FINAL (gates G1-G9 verdes, regresión) + REVISION-FINAL.md y F2-NOTAS §9
Via: Claude Code

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015AJuJLbhFstHGHc1VA1PnR
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/mobile-bar-business-plan/mobile-bar-financial-projections.xlsx
+++ b/astro-site/public/dl/mobile-bar-business-plan/mobile-bar-financial-projections.xlsx
@@ -717,7 +717,7 @@
     <row r="2" ht="59.75" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Change the GREEN cells: the rest of the workbook recalculates on its own. Expense items are typed on their own tab (also in green) and are not repeated here. Amounts are in your currency.</t>
+          <t>Change the GREEN cells: the rest of the workbook recalculates on its own. Expense items are typed on their own tab (also in green) and are not repeated here. Amounts are in US dollars (or your own currency).</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Price per guest for a dry hire event (you supply the alcohol; we bring the bar, the bartenders and everything else), EXCL. sales tax and excl. alcohol: the bar package plus add-ons, with bartenders, mixers, garnishes, ice and cups included, the service charge in and the voluntary gratuity out. Price per guest incl. sales tax = this value × (1 + your sales tax rate). The example sits inside the per-guest pricing range in the benchmarks table on the "Instructions" tab; the Pricing Calculator builds your quote from your own costs and hours: divide its subtotal by the billable guests to bring it here.</t>
+          <t>Price per guest for a dry hire event (your client buys the alcohol; you bring the bar, the bartenders and everything else), EXCL. sales tax and excl. alcohol: the bar package plus add-ons, with bartenders, mixers, garnishes, ice and cups included, the service charge in and the voluntary gratuity out. Price per guest incl. sales tax = this value × (1 + your sales tax rate). At 95 guests, 14 per guest gives 1,330 per event: above Check Cherry's $750 median and in the upper quarter (the middle half runs $450-$1,275; see the benchmarks table on the "Instructions" tab). the Pricing Calculator builds your quote from your own costs and hours: divide its subtotal by the billable guests to bring it here.</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Card fees on total sales. Hosts and planners mostly pay by card, with some ACH or check from companies, which lowers the cost. The example (2.5%) is a blended rate: a percentage plus a per-transaction fee, which weighs more on small deposits. Check your processor's statement and enter your effective rate (Kit estimate).</t>
+          <t>Card fees on total sales. Hosts and planners mostly pay by card, with some ACH or check from companies, which lowers the cost. The example (3%) is a blended rate: a percentage plus a per-transaction fee, which weighs more on small deposits. Check your processor's statement and enter your effective rate (Kit estimate).</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>FICA (Social Security 6.2% + Medicare 1.45%) + federal and state unemployment taxes (FUTA / SUTA) + workers' comp. The example uses a lean 10% with no benefits; the benchmarks table on "Instructions" gives the bartender wage. Ask your payroll provider and carrier for your rate.</t>
+          <t>FICA (Social Security 6.2% + Medicare 1.45%) + federal and state unemployment taxes (FUTA / SUTA). Workers' comp is in the insurance line. The example uses a lean 10% with no benefits; ask your payroll provider for your rate.</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Yearly insurance: general liability plus liquor liability (Kit estimate 600-1,000), commercial auto covering the trailer (about 1,800), workers' comp for your W-2 bartenders (about 1,000) and equipment cover (about 300). Venues ask for a COI naming them as additional insured, and general liability plus liquor liability starts around 550 a year (insurancecanopy.com). The total is a Kit estimate: get quotes before you fix it.</t>
+          <t>Yearly insurance: general liability plus liquor liability (Kit estimate 600-1,000), commercial auto covering the trailer (about 1,800), workers' comp for your W-2 bartenders (about 1,000) and equipment coverage (about 300). Venues ask for a COI naming them as additional insured, and general liability plus liquor liability start around $550 a year, bundled (insurancecanopy.com). The total is a Kit estimate: get quotes before you fix it.</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Sales tax rate on alcohol to go</t>
+          <t>Sales tax rate on alcohol sold (licensed only)</t>
         </is>
       </c>
       <c r="B40" s="63" t="n">
@@ -1717,7 +1717,7 @@
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
         <is>
-          <t>Bar trailer, used (6 x 12 ft cargo / concession or horse trailer)</t>
+          <t>Bar trailer, used (6 x 12 ft (1.8 x 3.7 m) cargo / concession or horse trailer)</t>
         </is>
       </c>
       <c r="B7" s="49" t="n">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>A used bar trailer (6 x 12 ft cargo, concession or horse trailer) that you convert. The tow vehicle is yours, so it costs 0 in the plan: if you do not have one, a used pickup is an extra purchase starting around 10,000 (checkcherry.com). Prices vary a lot with size and condition, so get several quotes.</t>
+          <t>A used bar trailer (6 x 12 ft (1.8 x 3.7 m) cargo, concession or horse trailer) that you convert. The tow vehicle is yours, so it costs 0 in the plan: if you do not have one, a used pickup is an extra purchase starting around $10,000 (checkcherry.com). Prices vary a lot with size and condition, so get several quotes.</t>
         </is>
       </c>
       <c r="E7" s="31" t="inlineStr">
@@ -6386,22 +6386,22 @@
     <row r="49" ht="45" customHeight="1">
       <c r="A49" s="58" t="inlineStr">
         <is>
-          <t>Fuel and miscellaneous</t>
+          <t>Miscellaneous event costs</t>
         </is>
       </c>
       <c r="B49" s="58" t="inlineStr">
         <is>
-          <t>Fuel and a miscellaneous line typed in among the fixed costs</t>
+          <t>A miscellaneous line typed in among the fixed costs</t>
         </is>
       </c>
       <c r="C49" s="58" t="inlineStr">
         <is>
-          <t>One percentage of sales, treated as a variable cost</t>
+          <t>A percentage of sales, treated as a variable cost; tow vehicle and trailer fuel has its own fixed line</t>
         </is>
       </c>
       <c r="D49" s="17" t="inlineStr">
         <is>
-          <t>Fuel rises and falls with the number of events you work: putting it among the fixed costs distorts the break-even.</t>
+          <t>Extra ice, last-minute mixers and venue parking rise and fall with the number of events: among the fixed costs they would distort the break-even.</t>
         </is>
       </c>
     </row>

</xml_diff>